<commit_message>
Make the dataset template's example rows a healthy module, and say how to fill the file in
The five example rows were hand-written and exceeded the generic module's short-circuit current and
maximum power, so the template scored Abnormal. They now sit just under the twin's maximum power,
and tests check both the built-in rows and the shipped template files score Normal.

The simple manual gains a section on filling a dataset in properly, and a troubleshooting row.
</commit_message>
<xml_diff>
--- a/docs/templates/pvysics-dataset-template.xlsx
+++ b/docs/templates/pvysics-dataset-template.xlsx
@@ -58,10 +58,10 @@
         <v>31.8</v>
       </c>
       <c r="D2">
-        <v>29.1</v>
+        <v>29.0</v>
       </c>
       <c r="E2">
-        <v>6.02</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="3">
@@ -77,10 +77,10 @@
         <v>31.9</v>
       </c>
       <c r="D3">
-        <v>29.1</v>
+        <v>29.0</v>
       </c>
       <c r="E3">
-        <v>6.08</v>
+        <v>5.15</v>
       </c>
     </row>
     <row r="4">
@@ -99,7 +99,7 @@
         <v>29.0</v>
       </c>
       <c r="E4">
-        <v>6.13</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="5">
@@ -118,7 +118,7 @@
         <v>29.0</v>
       </c>
       <c r="E5">
-        <v>6.19</v>
+        <v>5.25</v>
       </c>
     </row>
     <row r="6">
@@ -137,7 +137,7 @@
         <v>29.0</v>
       </c>
       <c r="E6">
-        <v>6.25</v>
+        <v>5.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>